<commit_message>
added colony and probio data
</commit_message>
<xml_diff>
--- a/Sample_Data/Probiotic_Field_Trials.xlsx
+++ b/Sample_Data/Probiotic_Field_Trials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/feliciaaronson/Documents/GitHub/SAN_CORDAP/Sample_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BD88110-A7DA-3E40-BFD3-CDA2C66AE40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49C5231-FD64-E84D-96D6-C019D15F5B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1400" windowWidth="27640" windowHeight="16680" xr2:uid="{6A471E7E-6015-6B4B-9FEA-6BF2E41A1795}"/>
+    <workbookView xWindow="7380" yWindow="1400" windowWidth="21760" windowHeight="16680" xr2:uid="{6A471E7E-6015-6B4B-9FEA-6BF2E41A1795}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="29">
   <si>
     <t>Transect</t>
   </si>
@@ -117,6 +117,12 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>ELARBOL</t>
+  </si>
+  <si>
+    <t>Healthy</t>
   </si>
 </sst>
 </file>
@@ -498,13 +504,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773221E2-9061-694C-B9CA-CA59BFE8DDED}">
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="7" width="17" customWidth="1"/>
     <col min="8" max="8" width="21.33203125" customWidth="1"/>
     <col min="9" max="9" width="19.6640625" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="10" max="10" width="31" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
@@ -1714,7 +1720,7 @@
         <v>18</v>
       </c>
       <c r="J39">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
@@ -1775,6 +1781,555 @@
         <v>21</v>
       </c>
       <c r="J41" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>27</v>
+      </c>
+      <c r="B42">
+        <v>5</v>
+      </c>
+      <c r="C42">
+        <v>19</v>
+      </c>
+      <c r="D42" t="s">
+        <v>15</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" t="s">
+        <v>12</v>
+      </c>
+      <c r="H42" t="s">
+        <v>17</v>
+      </c>
+      <c r="I42" t="s">
+        <v>18</v>
+      </c>
+      <c r="J42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>27</v>
+      </c>
+      <c r="B43">
+        <v>5</v>
+      </c>
+      <c r="C43">
+        <v>21</v>
+      </c>
+      <c r="D43" t="s">
+        <v>15</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" t="s">
+        <v>10</v>
+      </c>
+      <c r="G43" t="s">
+        <v>22</v>
+      </c>
+      <c r="H43" t="s">
+        <v>28</v>
+      </c>
+      <c r="I43" t="s">
+        <v>28</v>
+      </c>
+      <c r="J43" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>27</v>
+      </c>
+      <c r="B44">
+        <v>5</v>
+      </c>
+      <c r="C44">
+        <v>22</v>
+      </c>
+      <c r="D44" t="s">
+        <v>15</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G44" t="s">
+        <v>20</v>
+      </c>
+      <c r="H44" t="s">
+        <v>28</v>
+      </c>
+      <c r="I44" t="s">
+        <v>28</v>
+      </c>
+      <c r="J44" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>27</v>
+      </c>
+      <c r="B45">
+        <v>5</v>
+      </c>
+      <c r="C45">
+        <v>23</v>
+      </c>
+      <c r="D45" t="s">
+        <v>15</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G45" t="s">
+        <v>20</v>
+      </c>
+      <c r="H45" t="s">
+        <v>28</v>
+      </c>
+      <c r="I45" t="s">
+        <v>28</v>
+      </c>
+      <c r="J45" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>27</v>
+      </c>
+      <c r="B46">
+        <v>5</v>
+      </c>
+      <c r="C46">
+        <v>24</v>
+      </c>
+      <c r="D46" t="s">
+        <v>15</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G46" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" t="s">
+        <v>17</v>
+      </c>
+      <c r="I46" t="s">
+        <v>18</v>
+      </c>
+      <c r="J46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>27</v>
+      </c>
+      <c r="B47">
+        <v>5</v>
+      </c>
+      <c r="C47">
+        <v>29</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G47" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" t="s">
+        <v>28</v>
+      </c>
+      <c r="I47" t="s">
+        <v>28</v>
+      </c>
+      <c r="J47" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>27</v>
+      </c>
+      <c r="B48">
+        <v>5</v>
+      </c>
+      <c r="C48">
+        <v>31</v>
+      </c>
+      <c r="D48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F48" t="s">
+        <v>10</v>
+      </c>
+      <c r="G48" t="s">
+        <v>22</v>
+      </c>
+      <c r="H48" t="s">
+        <v>28</v>
+      </c>
+      <c r="I48" t="s">
+        <v>28</v>
+      </c>
+      <c r="J48" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>27</v>
+      </c>
+      <c r="B49">
+        <v>5</v>
+      </c>
+      <c r="C49">
+        <v>32</v>
+      </c>
+      <c r="D49" t="s">
+        <v>15</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G49" t="s">
+        <v>20</v>
+      </c>
+      <c r="H49" t="s">
+        <v>28</v>
+      </c>
+      <c r="I49" t="s">
+        <v>28</v>
+      </c>
+      <c r="J49" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>27</v>
+      </c>
+      <c r="B50">
+        <v>5</v>
+      </c>
+      <c r="C50">
+        <v>33</v>
+      </c>
+      <c r="D50" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F50" t="s">
+        <v>10</v>
+      </c>
+      <c r="G50" t="s">
+        <v>22</v>
+      </c>
+      <c r="H50" t="s">
+        <v>28</v>
+      </c>
+      <c r="I50" t="s">
+        <v>28</v>
+      </c>
+      <c r="J50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>27</v>
+      </c>
+      <c r="B51">
+        <v>5</v>
+      </c>
+      <c r="C51">
+        <v>34</v>
+      </c>
+      <c r="D51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G51" t="s">
+        <v>12</v>
+      </c>
+      <c r="H51" t="s">
+        <v>17</v>
+      </c>
+      <c r="I51" t="s">
+        <v>18</v>
+      </c>
+      <c r="J51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B52">
+        <v>5</v>
+      </c>
+      <c r="C52">
+        <v>35</v>
+      </c>
+      <c r="D52" t="s">
+        <v>15</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F52" t="s">
+        <v>10</v>
+      </c>
+      <c r="G52" t="s">
+        <v>11</v>
+      </c>
+      <c r="H52" t="s">
+        <v>17</v>
+      </c>
+      <c r="I52" t="s">
+        <v>18</v>
+      </c>
+      <c r="J52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>27</v>
+      </c>
+      <c r="B53">
+        <v>5</v>
+      </c>
+      <c r="C53">
+        <v>43</v>
+      </c>
+      <c r="D53" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F53" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53" t="s">
+        <v>22</v>
+      </c>
+      <c r="H53" t="s">
+        <v>28</v>
+      </c>
+      <c r="I53" t="s">
+        <v>28</v>
+      </c>
+      <c r="J53" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>27</v>
+      </c>
+      <c r="B54">
+        <v>5</v>
+      </c>
+      <c r="C54">
+        <v>44</v>
+      </c>
+      <c r="D54" t="s">
+        <v>15</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G54" t="s">
+        <v>20</v>
+      </c>
+      <c r="H54" t="s">
+        <v>28</v>
+      </c>
+      <c r="I54" t="s">
+        <v>28</v>
+      </c>
+      <c r="J54" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>27</v>
+      </c>
+      <c r="B55">
+        <v>5</v>
+      </c>
+      <c r="C55">
+        <v>89</v>
+      </c>
+      <c r="D55" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F55" t="s">
+        <v>10</v>
+      </c>
+      <c r="G55" t="s">
+        <v>11</v>
+      </c>
+      <c r="H55" t="s">
+        <v>17</v>
+      </c>
+      <c r="I55" t="s">
+        <v>17</v>
+      </c>
+      <c r="J55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>27</v>
+      </c>
+      <c r="B56">
+        <v>5</v>
+      </c>
+      <c r="C56">
+        <v>90</v>
+      </c>
+      <c r="D56" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G56" t="s">
+        <v>12</v>
+      </c>
+      <c r="H56" t="s">
+        <v>17</v>
+      </c>
+      <c r="I56" t="s">
+        <v>17</v>
+      </c>
+      <c r="J56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>27</v>
+      </c>
+      <c r="B57">
+        <v>5</v>
+      </c>
+      <c r="C57">
+        <v>91</v>
+      </c>
+      <c r="D57" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F57" t="s">
+        <v>10</v>
+      </c>
+      <c r="G57" t="s">
+        <v>11</v>
+      </c>
+      <c r="H57" t="s">
+        <v>17</v>
+      </c>
+      <c r="I57" t="s">
+        <v>17</v>
+      </c>
+      <c r="J57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>27</v>
+      </c>
+      <c r="B58">
+        <v>5</v>
+      </c>
+      <c r="C58">
+        <v>92</v>
+      </c>
+      <c r="D58" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G58" t="s">
+        <v>12</v>
+      </c>
+      <c r="H58" t="s">
+        <v>17</v>
+      </c>
+      <c r="I58" t="s">
+        <v>17</v>
+      </c>
+      <c r="J58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B59">
+        <v>5</v>
+      </c>
+      <c r="C59">
+        <v>28</v>
+      </c>
+      <c r="D59" t="s">
+        <v>15</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" t="s">
+        <v>10</v>
+      </c>
+      <c r="G59" t="s">
+        <v>22</v>
+      </c>
+      <c r="H59" t="s">
+        <v>28</v>
+      </c>
+      <c r="I59" t="s">
+        <v>28</v>
+      </c>
+      <c r="J59" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added sample information from valeria (Probiotic_Field_Trials_052926 google drive doc)
</commit_message>
<xml_diff>
--- a/Sample_Data/Probiotic_Field_Trials.xlsx
+++ b/Sample_Data/Probiotic_Field_Trials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/feliciaaronson/Documents/GitHub/SAN_CORDAP/Sample_Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikea_ulrich/Documents/GitHub/SAN_CORDAP/Sample_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49C5231-FD64-E84D-96D6-C019D15F5B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2B0DF9B-5922-C848-AE9F-61E2D4AED178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7380" yWindow="1400" windowWidth="21760" windowHeight="16680" xr2:uid="{6A471E7E-6015-6B4B-9FEA-6BF2E41A1795}"/>
+    <workbookView xWindow="31480" yWindow="1620" windowWidth="32600" windowHeight="19700" xr2:uid="{6A471E7E-6015-6B4B-9FEA-6BF2E41A1795}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="54">
   <si>
     <t>Transect</t>
   </si>
@@ -123,6 +123,81 @@
   </si>
   <si>
     <t>Healthy</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Health_Status_042026</t>
+  </si>
+  <si>
+    <t>Lesion_Progression_042026(cm)</t>
+  </si>
+  <si>
+    <t>New_Lesions_042026</t>
+  </si>
+  <si>
+    <t>Notes_042026</t>
+  </si>
+  <si>
+    <t>Health_Status_062026</t>
+  </si>
+  <si>
+    <t>Lesion_Progression_062026(cm)</t>
+  </si>
+  <si>
+    <t>New_Lesions_062026</t>
+  </si>
+  <si>
+    <t>Notes_062026</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>New lesion, No progression from nail</t>
+  </si>
+  <si>
+    <t>Snail lesions</t>
+  </si>
+  <si>
+    <t>No nail</t>
+  </si>
+  <si>
+    <t>2 lesions</t>
+  </si>
+  <si>
+    <t>No disease observed</t>
+  </si>
+  <si>
+    <t>Fish bites</t>
+  </si>
+  <si>
+    <t>SCTLD and snail lesions</t>
+  </si>
+  <si>
+    <t>Not found/not retreated - the original tag was #45 on the map were wrong the number (#15) and the location</t>
+  </si>
+  <si>
+    <t>Stegastes bites</t>
+  </si>
+  <si>
+    <t>Missing tag, No progression from nail</t>
+  </si>
+  <si>
+    <t>Disease no SC</t>
+  </si>
+  <si>
+    <t>Yellow Band Disease</t>
+  </si>
+  <si>
+    <t>No active lesions</t>
+  </si>
+  <si>
+    <t>Many active lesions, no nail to mesaure</t>
   </si>
 </sst>
 </file>
@@ -504,7 +579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773221E2-9061-694C-B9CA-CA59BFE8DDED}">
-  <dimension ref="A1:R59"/>
+  <dimension ref="A1:U59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="7" width="17" customWidth="1"/>
@@ -513,7 +588,7 @@
     <col min="10" max="10" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -547,8 +622,38 @@
       <c r="K1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S1" t="s">
+        <v>35</v>
+      </c>
+      <c r="T1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -579,9 +684,20 @@
       <c r="J2">
         <v>0</v>
       </c>
-      <c r="R2" s="3"/>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L2">
+        <v>23042026</v>
+      </c>
+      <c r="M2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -610,9 +726,23 @@
       <c r="J3">
         <v>0</v>
       </c>
-      <c r="R3" s="3"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L3">
+        <v>23042026</v>
+      </c>
+      <c r="M3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -643,9 +773,35 @@
       <c r="J4">
         <v>0</v>
       </c>
-      <c r="R4" s="3"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L4">
+        <v>23042026</v>
+      </c>
+      <c r="M4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4">
+        <v>3062026</v>
+      </c>
+      <c r="R4" t="s">
+        <v>28</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4" t="s">
+        <v>38</v>
+      </c>
+      <c r="U4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -674,9 +830,35 @@
       <c r="J5">
         <v>0</v>
       </c>
-      <c r="R5" s="3"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L5">
+        <v>23042026</v>
+      </c>
+      <c r="M5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5">
+        <v>3062026</v>
+      </c>
+      <c r="R5" t="s">
+        <v>17</v>
+      </c>
+      <c r="S5" t="s">
+        <v>42</v>
+      </c>
+      <c r="T5" t="s">
+        <v>39</v>
+      </c>
+      <c r="U5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -707,9 +889,20 @@
       <c r="J6">
         <v>0.5</v>
       </c>
-      <c r="R6" s="3"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L6">
+        <v>23042026</v>
+      </c>
+      <c r="M6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -738,9 +931,23 @@
       <c r="J7">
         <v>0.5</v>
       </c>
-      <c r="R7" s="3"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L7">
+        <v>23042026</v>
+      </c>
+      <c r="M7" t="s">
+        <v>28</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7" t="s">
+        <v>38</v>
+      </c>
+      <c r="P7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -771,9 +978,35 @@
       <c r="J8">
         <v>0</v>
       </c>
-      <c r="R8" s="3"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L8">
+        <v>23042026</v>
+      </c>
+      <c r="M8" t="s">
+        <v>28</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q8">
+        <v>3062026</v>
+      </c>
+      <c r="R8" t="s">
+        <v>28</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8" t="s">
+        <v>38</v>
+      </c>
+      <c r="U8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -802,9 +1035,20 @@
       <c r="J9">
         <v>0</v>
       </c>
-      <c r="R9" s="3"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L9">
+        <v>23042026</v>
+      </c>
+      <c r="M9" t="s">
+        <v>28</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -835,9 +1079,35 @@
       <c r="J10">
         <v>0</v>
       </c>
-      <c r="R10" s="3"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L10">
+        <v>23042026</v>
+      </c>
+      <c r="M10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q10">
+        <v>3062026</v>
+      </c>
+      <c r="R10" t="s">
+        <v>17</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10" t="s">
+        <v>39</v>
+      </c>
+      <c r="U10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -865,8 +1135,26 @@
       <c r="J11">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L11">
+        <v>23042026</v>
+      </c>
+      <c r="M11" t="s">
+        <v>17</v>
+      </c>
+      <c r="N11">
+        <v>1.8</v>
+      </c>
+      <c r="O11" t="s">
+        <v>39</v>
+      </c>
+      <c r="P11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -894,8 +1182,20 @@
       <c r="J12" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L12">
+        <v>23042026</v>
+      </c>
+      <c r="M12" t="s">
+        <v>28</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -923,8 +1223,20 @@
       <c r="J13" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L13">
+        <v>23042026</v>
+      </c>
+      <c r="M13" t="s">
+        <v>28</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -956,7 +1268,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -988,7 +1300,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -1020,7 +1332,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -1048,8 +1360,20 @@
       <c r="J17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17">
+        <v>23042026</v>
+      </c>
+      <c r="M17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -1077,8 +1401,20 @@
       <c r="J18" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18">
+        <v>23042026</v>
+      </c>
+      <c r="M18" t="s">
+        <v>28</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -1110,7 +1446,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -1138,8 +1474,20 @@
       <c r="J20" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20">
+        <v>23042026</v>
+      </c>
+      <c r="M20" t="s">
+        <v>28</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -1171,7 +1519,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -1199,8 +1547,23 @@
       <c r="J22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22">
+        <v>22042026</v>
+      </c>
+      <c r="M22" t="s">
+        <v>17</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22" t="s">
+        <v>39</v>
+      </c>
+      <c r="P22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1231,8 +1594,35 @@
       <c r="J23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23">
+        <v>22042026</v>
+      </c>
+      <c r="M23" t="s">
+        <v>17</v>
+      </c>
+      <c r="N23">
+        <v>0.2</v>
+      </c>
+      <c r="O23" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q23">
+        <v>2062026</v>
+      </c>
+      <c r="R23" t="s">
+        <v>28</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -1260,8 +1650,23 @@
       <c r="J24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24">
+        <v>22042026</v>
+      </c>
+      <c r="M24" t="s">
+        <v>17</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24" t="s">
+        <v>39</v>
+      </c>
+      <c r="P24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1289,8 +1694,23 @@
       <c r="J25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25">
+        <v>22042026</v>
+      </c>
+      <c r="M25" t="s">
+        <v>17</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25" t="s">
+        <v>39</v>
+      </c>
+      <c r="P25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1321,8 +1741,32 @@
       <c r="J26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26">
+        <v>22042026</v>
+      </c>
+      <c r="M26" t="s">
+        <v>28</v>
+      </c>
+      <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q26">
+        <v>2062026</v>
+      </c>
+      <c r="R26" t="s">
+        <v>28</v>
+      </c>
+      <c r="S26">
+        <v>0</v>
+      </c>
+      <c r="T26" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -1350,8 +1794,23 @@
       <c r="J27">
         <v>5</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L27">
+        <v>22042026</v>
+      </c>
+      <c r="M27" t="s">
+        <v>17</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27" t="s">
+        <v>39</v>
+      </c>
+      <c r="P27" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -1382,8 +1841,35 @@
       <c r="J28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L28">
+        <v>22042026</v>
+      </c>
+      <c r="M28" t="s">
+        <v>28</v>
+      </c>
+      <c r="N28">
+        <v>0.3</v>
+      </c>
+      <c r="O28" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q28">
+        <v>2062026</v>
+      </c>
+      <c r="R28" t="s">
+        <v>50</v>
+      </c>
+      <c r="S28">
+        <v>0</v>
+      </c>
+      <c r="T28" t="s">
+        <v>38</v>
+      </c>
+      <c r="U28" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -1411,8 +1897,23 @@
       <c r="J29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L29">
+        <v>22042026</v>
+      </c>
+      <c r="M29" t="s">
+        <v>17</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29" t="s">
+        <v>39</v>
+      </c>
+      <c r="P29" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1446,8 +1947,20 @@
       <c r="K30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="Q30">
+        <v>2062026</v>
+      </c>
+      <c r="R30" t="s">
+        <v>28</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -1475,8 +1988,17 @@
       <c r="J31" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L31">
+        <v>22042026</v>
+      </c>
+      <c r="M31" t="s">
+        <v>28</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -1508,7 +2030,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -1536,8 +2058,20 @@
       <c r="J33" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L33">
+        <v>22042026</v>
+      </c>
+      <c r="M33" t="s">
+        <v>28</v>
+      </c>
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -1569,7 +2103,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -1597,8 +2131,20 @@
       <c r="J35" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L35">
+        <v>22042026</v>
+      </c>
+      <c r="M35" t="s">
+        <v>28</v>
+      </c>
+      <c r="N35">
+        <v>0</v>
+      </c>
+      <c r="O35" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -1630,7 +2176,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -1662,7 +2208,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>23</v>
       </c>
@@ -1690,8 +2236,20 @@
       <c r="J38" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L38">
+        <v>22042026</v>
+      </c>
+      <c r="M38" t="s">
+        <v>28</v>
+      </c>
+      <c r="N38">
+        <v>0</v>
+      </c>
+      <c r="O38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>23</v>
       </c>
@@ -1722,8 +2280,32 @@
       <c r="J39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L39">
+        <v>22042026</v>
+      </c>
+      <c r="M39" t="s">
+        <v>28</v>
+      </c>
+      <c r="N39">
+        <v>0</v>
+      </c>
+      <c r="O39" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q39">
+        <v>2062026</v>
+      </c>
+      <c r="R39" t="s">
+        <v>17</v>
+      </c>
+      <c r="S39">
+        <v>2.5</v>
+      </c>
+      <c r="T39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>23</v>
       </c>
@@ -1751,8 +2333,20 @@
       <c r="J40" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L40">
+        <v>22042026</v>
+      </c>
+      <c r="M40" t="s">
+        <v>28</v>
+      </c>
+      <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>23</v>
       </c>
@@ -1784,7 +2378,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>27</v>
       </c>
@@ -1813,7 +2407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>27</v>
       </c>
@@ -1845,7 +2439,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>27</v>
       </c>
@@ -1874,7 +2468,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>27</v>
       </c>
@@ -1903,7 +2497,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>27</v>
       </c>
@@ -1934,8 +2528,32 @@
       <c r="J46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L46">
+        <v>24022026</v>
+      </c>
+      <c r="M46" t="s">
+        <v>17</v>
+      </c>
+      <c r="N46">
+        <v>0.2</v>
+      </c>
+      <c r="Q46">
+        <v>6062026</v>
+      </c>
+      <c r="R46" t="s">
+        <v>17</v>
+      </c>
+      <c r="S46">
+        <v>0</v>
+      </c>
+      <c r="T46" t="s">
+        <v>38</v>
+      </c>
+      <c r="U46" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>27</v>
       </c>
@@ -1964,7 +2582,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>27</v>
       </c>
@@ -1996,7 +2614,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>27</v>
       </c>
@@ -2025,7 +2643,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>27</v>
       </c>
@@ -2057,7 +2675,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>27</v>
       </c>
@@ -2086,7 +2704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>27</v>
       </c>
@@ -2117,8 +2735,29 @@
       <c r="J52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L52">
+        <v>24022026</v>
+      </c>
+      <c r="M52" t="s">
+        <v>17</v>
+      </c>
+      <c r="N52">
+        <v>0.4</v>
+      </c>
+      <c r="Q52">
+        <v>6062026</v>
+      </c>
+      <c r="R52" t="s">
+        <v>17</v>
+      </c>
+      <c r="S52">
+        <v>0</v>
+      </c>
+      <c r="T52" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>27</v>
       </c>
@@ -2150,7 +2789,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>27</v>
       </c>
@@ -2179,7 +2818,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>27</v>
       </c>
@@ -2210,8 +2849,35 @@
       <c r="J55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L55">
+        <v>24022026</v>
+      </c>
+      <c r="M55" t="s">
+        <v>28</v>
+      </c>
+      <c r="N55">
+        <v>0.4</v>
+      </c>
+      <c r="O55" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q55">
+        <v>6062026</v>
+      </c>
+      <c r="R55" t="s">
+        <v>17</v>
+      </c>
+      <c r="S55">
+        <v>0</v>
+      </c>
+      <c r="T55" t="s">
+        <v>38</v>
+      </c>
+      <c r="U55" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>27</v>
       </c>
@@ -2240,7 +2906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>27</v>
       </c>
@@ -2271,8 +2937,29 @@
       <c r="J57">
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L57">
+        <v>24022026</v>
+      </c>
+      <c r="M57" t="s">
+        <v>17</v>
+      </c>
+      <c r="N57" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q57">
+        <v>6062026</v>
+      </c>
+      <c r="R57" t="s">
+        <v>17</v>
+      </c>
+      <c r="S57">
+        <v>0</v>
+      </c>
+      <c r="T57" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>27</v>
       </c>
@@ -2301,7 +2988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>27</v>
       </c>

</xml_diff>